<commit_message>
updated gui in view records
updated gui, fixed the lacking space or name cut off in view records where if emplyee name is long the name will get cut off
</commit_message>
<xml_diff>
--- a/logs/login_logout_log.xlsx
+++ b/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -646,6 +646,35 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2024-11-16 08:07:52</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>user1</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2024-11-16 08:07:52</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
updated gui and session
</commit_message>
<xml_diff>
--- a/logs/login_logout_log.xlsx
+++ b/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -646,6 +646,35 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2024-11-16 08:27:01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>user1</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2024-11-16 08:27:01</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
added scrollbar to view employee record
added a copy of the previous view employee ui; new copy has scroll bar capabilities
</commit_message>
<xml_diff>
--- a/logs/login_logout_log.xlsx
+++ b/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -675,6 +675,40 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2024-11-16 21:40:51</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2024-11-16 22:50:06</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
added filter and updated pdf save loc
added filtering to the dashboard and updated the explicit folder save location in addnewemp module to dynamic
</commit_message>
<xml_diff>
--- a/logs/login_logout_log.xlsx
+++ b/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1048,6 +1048,429 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:22:14</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:22:50</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:24:55</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:25:09</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:31:43</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:32:26</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:33:47</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:34:12</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:37:25</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:37:40</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:38:01</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:38:09</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:41:41</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:41:51</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:42:25</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:42:37</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:42:59</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:43:10</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:43:32</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:45:11</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:45:31</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:46:23</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:46:46</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:48:16</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:48:29</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:49:34</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:49:49</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:53:52</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2024-11-18 17:54:42</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
updated archive.py, added edit_emp.py
updated archive.py to get the id of the employee, added edit_emp and fixed some ui elements
</commit_message>
<xml_diff>
--- a/logs/login_logout_log.xlsx
+++ b/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1500,6 +1500,168 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2024-11-19 18:59:07</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2024-11-19 18:59:48</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2024-11-19 19:02:04</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2024-11-19 19:02:13</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2024-11-19 19:05:15</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2024-11-19 19:05:34</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2024-11-19 19:07:00</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2024-11-19 19:08:04</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2024-11-19 19:08:28</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2024-11-19 19:09:09</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2024-11-19 19:20:35</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
continued working on displaying data
</commit_message>
<xml_diff>
--- a/logs/login_logout_log.xlsx
+++ b/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C108"/>
+  <dimension ref="A1:C111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2032,6 +2032,57 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2024-11-19 21:46:43</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2024-11-19 21:55:32</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2024-11-19 22:28:41</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fixed some things in dashboard.py and regarding with the session bugs are fixed (probably?)
</commit_message>
<xml_diff>
--- a/logs/login_logout_log.xlsx
+++ b/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -959,6 +959,23 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2024-11-19 22:31:55</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
automatic log out of session when program directly closed
</commit_message>
<xml_diff>
--- a/logs/login_logout_log.xlsx
+++ b/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1034,6 +1034,81 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2024-11-19 23:00:34</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2024-11-19 23:02:17</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2024-11-19 23:03:49</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2024-11-19 23:04:54</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2024-11-19 23:04:58</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Working nonfilipino part 2
working nani ang nonfilipino ang passport mu gawas
</commit_message>
<xml_diff>
--- a/logs/login_logout_log.xlsx
+++ b/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1350,6 +1350,105 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2024-11-20 14:26:28</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2024-11-20 14:26:55</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2024-11-20 14:28:34</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2024-11-20 14:29:25</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2024-11-20 14:31:18</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2024-11-20 14:35:23</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2024-11-20 14:36:09</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
just pushing nothing change
</commit_message>
<xml_diff>
--- a/logs/login_logout_log.xlsx
+++ b/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1449,6 +1449,35 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2024-11-20 15:00:48</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2024-11-20 15:01:53</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
added image functionality to add and view only
</commit_message>
<xml_diff>
--- a/logs/login_logout_log.xlsx
+++ b/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1749,6 +1749,267 @@
         </is>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2024-11-24 08:19:49</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2024-11-24 08:20:05</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2024-11-24 08:20:50</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2024-11-24 08:21:01</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2024-11-24 08:26:59</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2024-11-24 08:27:12</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2024-11-24 08:32:38</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2024-11-24 08:33:04</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2024-11-24 08:35:33</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2024-11-24 08:35:47</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2024-11-24 08:38:35</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2024-11-24 08:38:40</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2024-11-24 08:39:07</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2024-11-24 08:39:13</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2024-11-24 08:39:26</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2024-11-24 08:39:33</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2024-11-24 08:40:10</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2024-11-24 08:40:19</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
added new ui files
</commit_message>
<xml_diff>
--- a/logs/login_logout_log.xlsx
+++ b/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2039,6 +2039,35 @@
         </is>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2024-12-01 08:06:14</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2024-12-01 08:07:23</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
updated ui based on canlas changes
added canlas ui, has issues on dark mode themes
</commit_message>
<xml_diff>
--- a/logs/login_logout_log.xlsx
+++ b/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C106"/>
+  <dimension ref="A1:C121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2068,6 +2068,226 @@
         </is>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2024-12-01 08:11:14</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2024-12-01 08:12:06</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2024-12-01 08:12:10</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2024-12-01 08:12:44</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2024-12-01 08:13:27</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2024-12-01 08:13:30</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2024-12-01 08:13:54</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2024-12-01 08:13:58</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2024-12-01 08:14:54</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2024-12-01 08:15:47</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2024-12-01 08:17:18</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2024-12-01 08:20:16</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2024-12-01 08:20:21</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2024-12-01 08:22:38</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2024-12-01 08:22:56</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
connected salary window to view
</commit_message>
<xml_diff>
--- a/logs/login_logout_log.xlsx
+++ b/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C170"/>
+  <dimension ref="A1:C174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3001,6 +3001,64 @@
         </is>
       </c>
     </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2024-12-12 12:58:52</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2024-12-12 12:59:02</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2024-12-12 13:00:58</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2024-12-12 13:01:31</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
added spouse name to edit
</commit_message>
<xml_diff>
--- a/logs/login_logout_log.xlsx
+++ b/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C174"/>
+  <dimension ref="A1:C178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3059,6 +3059,64 @@
         </is>
       </c>
     </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2024-12-12 13:05:55</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2024-12-12 13:14:18</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2024-12-12 13:14:52</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2024-12-12 13:15:35</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
updated edit, added children view
</commit_message>
<xml_diff>
--- a/logs/login_logout_log.xlsx
+++ b/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C178"/>
+  <dimension ref="A1:C188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3117,6 +3117,151 @@
         </is>
       </c>
     </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2024-12-12 13:22:34</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2024-12-12 13:22:52</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2024-12-12 13:23:24</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2024-12-12 13:23:31</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2024-12-12 13:23:48</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2024-12-12 13:24:04</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2024-12-12 13:24:53</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2024-12-12 13:25:11</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2024-12-12 13:25:56</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2024-12-12 13:26:12</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
updated family in edit
</commit_message>
<xml_diff>
--- a/logs/login_logout_log.xlsx
+++ b/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C188"/>
+  <dimension ref="A1:C262"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3262,6 +3262,1084 @@
         </is>
       </c>
     </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:18:49</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:19:48</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:21:16</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:24:02</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:25:10</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:25:24</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:27:37</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:27:45</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:28:38</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:28:55</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:29:43</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:29:52</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:37:41</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:39:01</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:40:33</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:43:58</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:44:35</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:44:40</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:45:20</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:45:39</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:53:15</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:54:59</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:55:04</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:55:34</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:56:40</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:57:11</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:57:41</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:58:31</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:59:08</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:00:24</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:00:35</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:02:34</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:02:38</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:02:56</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:03:11</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:06:14</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:06:53</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:11:09</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:11:36</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:17:26</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:17:48</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:22:13</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:24:39</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:25:20</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:26:57</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:27:23</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:29:33</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:29:47</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:30:58</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:31:20</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:31:55</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:32:33</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:36:53</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:37:29</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:38:30</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:38:44</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:41:44</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:41:58</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:43:00</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:43:08</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:43:17</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:43:54</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:44:07</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:44:38</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:48:45</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:49:38</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:51:40</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:52:59</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:58:09</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:58:25</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:58:46</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2024-12-12 16:59:22</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2024-12-12 17:10:32</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2024-12-12 17:10:53</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
added spouse, sibling and crime
</commit_message>
<xml_diff>
--- a/logs/login_logout_log.xlsx
+++ b/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C361"/>
+  <dimension ref="A1:C377"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5778,6 +5778,238 @@
         </is>
       </c>
     </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2024-12-12 22:53:12</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2024-12-12 22:53:51</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2024-12-12 23:07:14</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2024-12-12 23:07:47</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2024-12-12 23:15:19</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2024-12-12 23:15:28</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2024-12-12 23:18:42</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2024-12-12 23:19:18</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2024-12-12 23:24:27</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2024-12-12 23:24:51</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2024-12-12 23:25:04</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2024-12-12 23:25:26</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2024-12-12 23:27:07</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2024-12-12 23:27:19</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2024-12-12 23:27:33</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2024-12-12 23:27:55</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
updated adding of government exams
</commit_message>
<xml_diff>
--- a/logs/login_logout_log.xlsx
+++ b/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C377"/>
+  <dimension ref="A1:C388"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6010,6 +6010,168 @@
         </is>
       </c>
     </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2024-12-13 07:52:31</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2024-12-13 07:53:42</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2024-12-13 08:01:05</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2024-12-13 08:02:33</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2024-12-13 08:07:41</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2024-12-13 08:09:03</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2024-12-13 08:09:20</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2024-12-13 08:10:30</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2024-12-13 08:13:27</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2024-12-13 08:15:33</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2024-12-13 08:16:39</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
updated edit and view module
</commit_message>
<xml_diff>
--- a/logs/login_logout_log.xlsx
+++ b/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C388"/>
+  <dimension ref="A1:C414"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6172,6 +6172,383 @@
         </is>
       </c>
     </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2024-12-13 09:27:57</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2024-12-13 09:28:17</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2024-12-13 09:29:27</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2024-12-13 09:37:36</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2024-12-13 09:57:10</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2024-12-13 09:58:08</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2024-12-13 10:05:14</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2024-12-13 10:06:02</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2024-12-13 10:13:18</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2024-12-13 10:13:31</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2024-12-13 10:15:57</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2024-12-13 10:16:18</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2024-12-13 10:20:24</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2024-12-13 10:20:35</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2024-12-13 10:20:47</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2024-12-13 10:23:14</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2024-12-13 10:24:02</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2024-12-13 10:25:07</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2024-12-13 10:26:01</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2024-12-13 10:26:17</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>2024-12-13 10:27:59</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2024-12-13 10:28:21</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>2024-12-13 10:30:38</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>2024-12-13 10:30:54</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>2024-12-13 10:33:23</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>2024-12-13 10:33:48</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
updated edit - 99%
</commit_message>
<xml_diff>
--- a/logs/login_logout_log.xlsx
+++ b/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C451"/>
+  <dimension ref="A1:C465"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7088,6 +7088,209 @@
         </is>
       </c>
     </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>2024-12-13 12:03:02</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>2024-12-13 12:11:34</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>2024-12-13 12:21:23</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>2024-12-13 12:23:11</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>2024-12-13 12:24:03</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>2024-12-13 12:24:38</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>2024-12-13 12:28:09</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>2024-12-13 12:28:34</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>2024-12-13 12:41:08</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>2024-12-13 12:43:58</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>2024-12-13 12:45:54</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>2024-12-13 12:46:08</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>2024-12-13 12:46:23</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>2024-12-13 12:46:46</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>